<commit_message>
Fix OpenAI API call: use chat.completions.create instead of invalid responses.create
</commit_message>
<xml_diff>
--- a/TestURL.xlsx
+++ b/TestURL.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tdworldwide-my.sharepoint.com/personal/t450877l_tdsynnex_com/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tdworldwide-my.sharepoint.com/personal/t450877l_tdsynnex_com/Documents/Documents/Projects/domain-recon/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BD50A00B-0378-4FDF-B622-978A821E4665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{BD50A00B-0378-4FDF-B622-978A821E4665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CEFA02B7-E149-404B-9C72-7F7794A751D8}"/>
   <bookViews>
-    <workbookView xWindow="-29976" yWindow="-1728" windowWidth="17712" windowHeight="12120" xr2:uid="{EBE2A85B-4012-4CF4-9014-38BE75861ECF}"/>
+    <workbookView xWindow="29760" yWindow="960" windowWidth="21600" windowHeight="11235" xr2:uid="{EBE2A85B-4012-4CF4-9014-38BE75861ECF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>google.com</t>
   </si>
@@ -60,6 +60,45 @@
   </si>
   <si>
     <t>internal-check.localhost</t>
+  </si>
+  <si>
+    <t>amazon.com</t>
+  </si>
+  <si>
+    <t>github.com</t>
+  </si>
+  <si>
+    <t>linkedin.com</t>
+  </si>
+  <si>
+    <t>microsoft.com</t>
+  </si>
+  <si>
+    <t>sony.com</t>
+  </si>
+  <si>
+    <t>apple.com</t>
+  </si>
+  <si>
+    <t>tesla.com</t>
+  </si>
+  <si>
+    <t>chatgpt.com</t>
+  </si>
+  <si>
+    <t>claude.com</t>
+  </si>
+  <si>
+    <t>vercel.com</t>
+  </si>
+  <si>
+    <t>servicesolv.ca</t>
+  </si>
+  <si>
+    <t>demandsolv.ca</t>
+  </si>
+  <si>
+    <t>emj.ca</t>
   </si>
 </sst>
 </file>
@@ -455,7 +494,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6446E2C5-5B42-4063-9049-13DD48124620}">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.21875" customWidth="1"/>
@@ -494,6 +533,71 @@
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>